<commit_message>
Excel: ölçülmeyen Trends satırları açıkça işaretlendi
Trends sütunları yalnızca sayfada listelenen 30 başlık için doluydu; kalan 73
satırda hücreler boştu ve bu "veri bulunamadı" gibi okunuyordu. Oysa o
başlıklar için ölçüm hiç yapılmadı.

Boş hücreler "-" ile işaretlendi (Bölüm 15.2 placeholder dili), sayfaya iki
not satırı eklendi ve terim sözlüğüne iki madde girdi. Ayrım metinde açık:
"-" verinin bulunamadığını değil ölçümün yapılmadığını gösterir.
</commit_message>
<xml_diff>
--- a/ozdilekteyim-eylul-2026-arama-talebi.xlsx
+++ b/ozdilekteyim-eylul-2026-arama-talebi.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2318,11 +2318,31 @@
       <c r="H32" s="10" t="n">
         <v>0.2235649546827795</v>
       </c>
-      <c r="I32" s="4" t="n"/>
-      <c r="J32" s="4" t="n"/>
-      <c r="K32" s="4" t="n"/>
-      <c r="L32" s="4" t="inlineStr"/>
-      <c r="M32" s="4" t="n"/>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2360,11 +2380,31 @@
       <c r="H33" s="5" t="n">
         <v>-0.4527027027027027</v>
       </c>
-      <c r="I33" s="4" t="n"/>
-      <c r="J33" s="4" t="n"/>
-      <c r="K33" s="4" t="n"/>
-      <c r="L33" s="4" t="inlineStr"/>
-      <c r="M33" s="4" t="n"/>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2402,11 +2442,31 @@
       <c r="H34" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="4" t="n"/>
-      <c r="J34" s="4" t="n"/>
-      <c r="K34" s="4" t="n"/>
-      <c r="L34" s="4" t="inlineStr"/>
-      <c r="M34" s="4" t="n"/>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2444,11 +2504,31 @@
       <c r="H35" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="n"/>
-      <c r="L35" s="4" t="inlineStr"/>
-      <c r="M35" s="4" t="n"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2486,11 +2566,31 @@
       <c r="H36" s="5" t="n">
         <v>-0.1818181818181818</v>
       </c>
-      <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="n"/>
-      <c r="L36" s="4" t="inlineStr"/>
-      <c r="M36" s="4" t="n"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2528,11 +2628,31 @@
       <c r="H37" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="n"/>
-      <c r="K37" s="4" t="n"/>
-      <c r="L37" s="4" t="inlineStr"/>
-      <c r="M37" s="4" t="n"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N37" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2570,11 +2690,31 @@
       <c r="H38" s="5" t="n">
         <v>-0.1818181818181818</v>
       </c>
-      <c r="I38" s="4" t="n"/>
-      <c r="J38" s="4" t="n"/>
-      <c r="K38" s="4" t="n"/>
-      <c r="L38" s="4" t="inlineStr"/>
-      <c r="M38" s="4" t="n"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2612,11 +2752,31 @@
       <c r="H39" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="4" t="n"/>
-      <c r="J39" s="4" t="n"/>
-      <c r="K39" s="4" t="n"/>
-      <c r="L39" s="4" t="inlineStr"/>
-      <c r="M39" s="4" t="n"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2654,11 +2814,31 @@
       <c r="H40" s="5" t="n">
         <v>-0.3305785123966942</v>
       </c>
-      <c r="I40" s="4" t="n"/>
-      <c r="J40" s="4" t="n"/>
-      <c r="K40" s="4" t="n"/>
-      <c r="L40" s="4" t="inlineStr"/>
-      <c r="M40" s="4" t="n"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2696,11 +2876,31 @@
       <c r="H41" s="5" t="n">
         <v>-0.1818181818181818</v>
       </c>
-      <c r="I41" s="4" t="n"/>
-      <c r="J41" s="4" t="n"/>
-      <c r="K41" s="4" t="n"/>
-      <c r="L41" s="4" t="inlineStr"/>
-      <c r="M41" s="4" t="n"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2738,11 +2938,31 @@
       <c r="H42" s="10" t="n">
         <v>0.4944649446494465</v>
       </c>
-      <c r="I42" s="4" t="n"/>
-      <c r="J42" s="4" t="n"/>
-      <c r="K42" s="4" t="n"/>
-      <c r="L42" s="4" t="inlineStr"/>
-      <c r="M42" s="4" t="n"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2784,11 +3004,31 @@
       <c r="H43" s="5" t="n">
         <v>-0.182716049382716</v>
       </c>
-      <c r="I43" s="4" t="n"/>
-      <c r="J43" s="4" t="n"/>
-      <c r="K43" s="4" t="n"/>
-      <c r="L43" s="4" t="inlineStr"/>
-      <c r="M43" s="4" t="n"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2826,11 +3066,31 @@
       <c r="H44" s="5" t="n">
         <v>-0.182716049382716</v>
       </c>
-      <c r="I44" s="4" t="n"/>
-      <c r="J44" s="4" t="n"/>
-      <c r="K44" s="4" t="n"/>
-      <c r="L44" s="4" t="inlineStr"/>
-      <c r="M44" s="4" t="n"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N44" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2868,11 +3128,31 @@
       <c r="H45" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I45" s="4" t="n"/>
-      <c r="J45" s="4" t="n"/>
-      <c r="K45" s="4" t="n"/>
-      <c r="L45" s="4" t="inlineStr"/>
-      <c r="M45" s="4" t="n"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N45" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2910,11 +3190,31 @@
       <c r="H46" s="5" t="n">
         <v>-0.182716049382716</v>
       </c>
-      <c r="I46" s="4" t="n"/>
-      <c r="J46" s="4" t="n"/>
-      <c r="K46" s="4" t="n"/>
-      <c r="L46" s="4" t="inlineStr"/>
-      <c r="M46" s="4" t="n"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N46" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2952,11 +3252,31 @@
       <c r="H47" s="5" t="n">
         <v>-0.3313131313131313</v>
       </c>
-      <c r="I47" s="4" t="n"/>
-      <c r="J47" s="4" t="n"/>
-      <c r="K47" s="4" t="n"/>
-      <c r="L47" s="4" t="inlineStr"/>
-      <c r="M47" s="4" t="n"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N47" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -2994,11 +3314,31 @@
       <c r="H48" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I48" s="4" t="n"/>
-      <c r="J48" s="4" t="n"/>
-      <c r="K48" s="4" t="n"/>
-      <c r="L48" s="4" t="inlineStr"/>
-      <c r="M48" s="4" t="n"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M48" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N48" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3036,11 +3376,31 @@
       <c r="H49" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I49" s="4" t="n"/>
-      <c r="J49" s="4" t="n"/>
-      <c r="K49" s="4" t="n"/>
-      <c r="L49" s="4" t="inlineStr"/>
-      <c r="M49" s="4" t="n"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N49" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3078,11 +3438,31 @@
       <c r="H50" s="5" t="n">
         <v>-0.182716049382716</v>
       </c>
-      <c r="I50" s="4" t="n"/>
-      <c r="J50" s="4" t="n"/>
-      <c r="K50" s="4" t="n"/>
-      <c r="L50" s="4" t="inlineStr"/>
-      <c r="M50" s="4" t="n"/>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N50" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3120,11 +3500,31 @@
       <c r="H51" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
-      <c r="K51" s="4" t="n"/>
-      <c r="L51" s="4" t="inlineStr"/>
-      <c r="M51" s="4" t="n"/>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N51" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3162,11 +3562,31 @@
       <c r="H52" s="10" t="n">
         <v>0.2214022140221402</v>
       </c>
-      <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="n"/>
-      <c r="K52" s="4" t="n"/>
-      <c r="L52" s="4" t="inlineStr"/>
-      <c r="M52" s="4" t="n"/>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N52" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3208,11 +3628,31 @@
       <c r="H53" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I53" s="4" t="n"/>
-      <c r="J53" s="4" t="n"/>
-      <c r="K53" s="4" t="n"/>
-      <c r="L53" s="4" t="inlineStr"/>
-      <c r="M53" s="4" t="n"/>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M53" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N53" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3254,11 +3694,31 @@
       <c r="H54" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="n"/>
-      <c r="K54" s="4" t="n"/>
-      <c r="L54" s="4" t="inlineStr"/>
-      <c r="M54" s="4" t="n"/>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N54" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3300,11 +3760,31 @@
       <c r="H55" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I55" s="4" t="n"/>
-      <c r="J55" s="4" t="n"/>
-      <c r="K55" s="4" t="n"/>
-      <c r="L55" s="4" t="inlineStr"/>
-      <c r="M55" s="4" t="n"/>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N55" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3346,11 +3826,31 @@
       <c r="H56" s="5" t="n">
         <v>-0.1812688821752266</v>
       </c>
-      <c r="I56" s="4" t="n"/>
-      <c r="J56" s="4" t="n"/>
-      <c r="K56" s="4" t="n"/>
-      <c r="L56" s="4" t="inlineStr"/>
-      <c r="M56" s="4" t="n"/>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N56" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3388,11 +3888,31 @@
       <c r="H57" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I57" s="4" t="n"/>
-      <c r="J57" s="4" t="n"/>
-      <c r="K57" s="4" t="n"/>
-      <c r="L57" s="4" t="inlineStr"/>
-      <c r="M57" s="4" t="n"/>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N57" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3430,11 +3950,31 @@
       <c r="H58" s="5" t="n">
         <v>-0.1812688821752266</v>
       </c>
-      <c r="I58" s="4" t="n"/>
-      <c r="J58" s="4" t="n"/>
-      <c r="K58" s="4" t="n"/>
-      <c r="L58" s="4" t="inlineStr"/>
-      <c r="M58" s="4" t="n"/>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N58" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3472,11 +4012,31 @@
       <c r="H59" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I59" s="4" t="n"/>
-      <c r="J59" s="4" t="n"/>
-      <c r="K59" s="4" t="n"/>
-      <c r="L59" s="4" t="inlineStr"/>
-      <c r="M59" s="4" t="n"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M59" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N59" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3514,11 +4074,31 @@
       <c r="H60" s="5" t="n">
         <v>-0.1812688821752266</v>
       </c>
-      <c r="I60" s="4" t="n"/>
-      <c r="J60" s="4" t="n"/>
-      <c r="K60" s="4" t="n"/>
-      <c r="L60" s="4" t="inlineStr"/>
-      <c r="M60" s="4" t="n"/>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N60" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3556,11 +4136,31 @@
       <c r="H61" s="5" t="n">
         <v>-0.4525252525252526</v>
       </c>
-      <c r="I61" s="4" t="n"/>
-      <c r="J61" s="4" t="n"/>
-      <c r="K61" s="4" t="n"/>
-      <c r="L61" s="4" t="inlineStr"/>
-      <c r="M61" s="4" t="n"/>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N61" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3598,11 +4198,31 @@
       <c r="H62" s="5" t="n">
         <v>-0.1812688821752266</v>
       </c>
-      <c r="I62" s="4" t="n"/>
-      <c r="J62" s="4" t="n"/>
-      <c r="K62" s="4" t="n"/>
-      <c r="L62" s="4" t="inlineStr"/>
-      <c r="M62" s="4" t="n"/>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N62" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3640,11 +4260,31 @@
       <c r="H63" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I63" s="4" t="n"/>
-      <c r="J63" s="4" t="n"/>
-      <c r="K63" s="4" t="n"/>
-      <c r="L63" s="4" t="inlineStr"/>
-      <c r="M63" s="4" t="n"/>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N63" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3682,11 +4322,31 @@
       <c r="H64" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="n"/>
-      <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="inlineStr"/>
-      <c r="M64" s="4" t="n"/>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L64" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M64" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N64" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3724,11 +4384,31 @@
       <c r="H65" s="5" t="n">
         <v>-0.4525252525252526</v>
       </c>
-      <c r="I65" s="4" t="n"/>
-      <c r="J65" s="4" t="n"/>
-      <c r="K65" s="4" t="n"/>
-      <c r="L65" s="4" t="inlineStr"/>
-      <c r="M65" s="4" t="n"/>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L65" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M65" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N65" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3766,11 +4446,31 @@
       <c r="H66" s="5" t="n">
         <v>-0.3308641975308642</v>
       </c>
-      <c r="I66" s="4" t="n"/>
-      <c r="J66" s="4" t="n"/>
-      <c r="K66" s="4" t="n"/>
-      <c r="L66" s="4" t="inlineStr"/>
-      <c r="M66" s="4" t="n"/>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L66" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N66" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3808,11 +4508,31 @@
       <c r="H67" s="5" t="n">
         <v>-0.1812688821752266</v>
       </c>
-      <c r="I67" s="4" t="n"/>
-      <c r="J67" s="4" t="n"/>
-      <c r="K67" s="4" t="n"/>
-      <c r="L67" s="4" t="inlineStr"/>
-      <c r="M67" s="4" t="n"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N67" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3850,11 +4570,31 @@
       <c r="H68" s="5" t="n">
         <v>-0.1812688821752266</v>
       </c>
-      <c r="I68" s="4" t="n"/>
-      <c r="J68" s="4" t="n"/>
-      <c r="K68" s="4" t="n"/>
-      <c r="L68" s="4" t="inlineStr"/>
-      <c r="M68" s="4" t="n"/>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M68" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3892,11 +4632,31 @@
       <c r="H69" s="5" t="n">
         <v>-0.1812688821752266</v>
       </c>
-      <c r="I69" s="4" t="n"/>
-      <c r="J69" s="4" t="n"/>
-      <c r="K69" s="4" t="n"/>
-      <c r="L69" s="4" t="inlineStr"/>
-      <c r="M69" s="4" t="n"/>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N69" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3934,11 +4694,31 @@
       <c r="H70" s="10" t="n">
         <v>0.2207207207207207</v>
       </c>
-      <c r="I70" s="4" t="n"/>
-      <c r="J70" s="4" t="n"/>
-      <c r="K70" s="4" t="n"/>
-      <c r="L70" s="4" t="inlineStr"/>
-      <c r="M70" s="4" t="n"/>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L70" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M70" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N70" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -3976,11 +4756,31 @@
       <c r="H71" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I71" s="4" t="n"/>
-      <c r="J71" s="4" t="n"/>
-      <c r="K71" s="4" t="n"/>
-      <c r="L71" s="4" t="inlineStr"/>
-      <c r="M71" s="4" t="n"/>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K71" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L71" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M71" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N71" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4018,11 +4818,31 @@
       <c r="H72" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I72" s="4" t="n"/>
-      <c r="J72" s="4" t="n"/>
-      <c r="K72" s="4" t="n"/>
-      <c r="L72" s="4" t="inlineStr"/>
-      <c r="M72" s="4" t="n"/>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L72" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M72" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N72" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4064,11 +4884,31 @@
       <c r="H73" s="5" t="n">
         <v>-0.1808118081180812</v>
       </c>
-      <c r="I73" s="4" t="n"/>
-      <c r="J73" s="4" t="n"/>
-      <c r="K73" s="4" t="n"/>
-      <c r="L73" s="4" t="inlineStr"/>
-      <c r="M73" s="4" t="n"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N73" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4110,11 +4950,31 @@
       <c r="H74" s="5" t="n">
         <v>-0.1808118081180812</v>
       </c>
-      <c r="I74" s="4" t="n"/>
-      <c r="J74" s="4" t="n"/>
-      <c r="K74" s="4" t="n"/>
-      <c r="L74" s="4" t="inlineStr"/>
-      <c r="M74" s="4" t="n"/>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L74" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M74" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4152,11 +5012,31 @@
       <c r="H75" s="5" t="n">
         <v>-0.3293051359516616</v>
       </c>
-      <c r="I75" s="4" t="n"/>
-      <c r="J75" s="4" t="n"/>
-      <c r="K75" s="4" t="n"/>
-      <c r="L75" s="4" t="inlineStr"/>
-      <c r="M75" s="4" t="n"/>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L75" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M75" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N75" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4194,11 +5074,31 @@
       <c r="H76" s="5" t="n">
         <v>-0.1808118081180812</v>
       </c>
-      <c r="I76" s="4" t="n"/>
-      <c r="J76" s="4" t="n"/>
-      <c r="K76" s="4" t="n"/>
-      <c r="L76" s="4" t="inlineStr"/>
-      <c r="M76" s="4" t="n"/>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M76" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4236,11 +5136,31 @@
       <c r="H77" s="5" t="n">
         <v>-0.3293051359516616</v>
       </c>
-      <c r="I77" s="4" t="n"/>
-      <c r="J77" s="4" t="n"/>
-      <c r="K77" s="4" t="n"/>
-      <c r="L77" s="4" t="inlineStr"/>
-      <c r="M77" s="4" t="n"/>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L77" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M77" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N77" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4278,11 +5198,31 @@
       <c r="H78" s="5" t="n">
         <v>-0.3293051359516616</v>
       </c>
-      <c r="I78" s="4" t="n"/>
-      <c r="J78" s="4" t="n"/>
-      <c r="K78" s="4" t="n"/>
-      <c r="L78" s="4" t="inlineStr"/>
-      <c r="M78" s="4" t="n"/>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L78" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M78" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N78" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4320,11 +5260,31 @@
       <c r="H79" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I79" s="4" t="n"/>
-      <c r="J79" s="4" t="n"/>
-      <c r="K79" s="4" t="n"/>
-      <c r="L79" s="4" t="inlineStr"/>
-      <c r="M79" s="4" t="n"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L79" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M79" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N79" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4362,11 +5322,31 @@
       <c r="H80" s="5" t="n">
         <v>-0.3293051359516616</v>
       </c>
-      <c r="I80" s="4" t="n"/>
-      <c r="J80" s="4" t="n"/>
-      <c r="K80" s="4" t="n"/>
-      <c r="L80" s="4" t="inlineStr"/>
-      <c r="M80" s="4" t="n"/>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L80" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M80" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N80" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4404,11 +5384,31 @@
       <c r="H81" s="5" t="n">
         <v>-0.1808118081180812</v>
       </c>
-      <c r="I81" s="4" t="n"/>
-      <c r="J81" s="4" t="n"/>
-      <c r="K81" s="4" t="n"/>
-      <c r="L81" s="4" t="inlineStr"/>
-      <c r="M81" s="4" t="n"/>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L81" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M81" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N81" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4446,11 +5446,31 @@
       <c r="H82" s="5" t="n">
         <v>-0.1808118081180812</v>
       </c>
-      <c r="I82" s="4" t="n"/>
-      <c r="J82" s="4" t="n"/>
-      <c r="K82" s="4" t="n"/>
-      <c r="L82" s="4" t="inlineStr"/>
-      <c r="M82" s="4" t="n"/>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L82" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M82" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N82" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4488,11 +5508,31 @@
       <c r="H83" s="5" t="n">
         <v>-0.3293051359516616</v>
       </c>
-      <c r="I83" s="4" t="n"/>
-      <c r="J83" s="4" t="n"/>
-      <c r="K83" s="4" t="n"/>
-      <c r="L83" s="4" t="inlineStr"/>
-      <c r="M83" s="4" t="n"/>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L83" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M83" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N83" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4530,11 +5570,31 @@
       <c r="H84" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="I84" s="4" t="n"/>
-      <c r="J84" s="4" t="n"/>
-      <c r="K84" s="4" t="n"/>
-      <c r="L84" s="4" t="inlineStr"/>
-      <c r="M84" s="4" t="n"/>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L84" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M84" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N84" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4572,11 +5632,31 @@
       <c r="H85" s="10" t="n">
         <v>0.2265193370165746</v>
       </c>
-      <c r="I85" s="4" t="n"/>
-      <c r="J85" s="4" t="n"/>
-      <c r="K85" s="4" t="n"/>
-      <c r="L85" s="4" t="inlineStr"/>
-      <c r="M85" s="4" t="n"/>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L85" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N85" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4618,11 +5698,31 @@
       <c r="H86" s="5" t="n">
         <v>-0.3321033210332103</v>
       </c>
-      <c r="I86" s="4" t="n"/>
-      <c r="J86" s="4" t="n"/>
-      <c r="K86" s="4" t="n"/>
-      <c r="L86" s="4" t="inlineStr"/>
-      <c r="M86" s="4" t="n"/>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L86" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M86" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N86" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4664,11 +5764,31 @@
       <c r="H87" s="5" t="n">
         <v>-0.3321033210332103</v>
       </c>
-      <c r="I87" s="4" t="n"/>
-      <c r="J87" s="4" t="n"/>
-      <c r="K87" s="4" t="n"/>
-      <c r="L87" s="4" t="inlineStr"/>
-      <c r="M87" s="4" t="n"/>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L87" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M87" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N87" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4710,11 +5830,31 @@
       <c r="H88" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I88" s="4" t="n"/>
-      <c r="J88" s="4" t="n"/>
-      <c r="K88" s="4" t="n"/>
-      <c r="L88" s="4" t="inlineStr"/>
-      <c r="M88" s="4" t="n"/>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L88" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M88" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N88" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4756,11 +5896,31 @@
       <c r="H89" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I89" s="4" t="n"/>
-      <c r="J89" s="4" t="n"/>
-      <c r="K89" s="4" t="n"/>
-      <c r="L89" s="4" t="inlineStr"/>
-      <c r="M89" s="4" t="n"/>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K89" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L89" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M89" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N89" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4798,11 +5958,31 @@
       <c r="H90" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I90" s="4" t="n"/>
-      <c r="J90" s="4" t="n"/>
-      <c r="K90" s="4" t="n"/>
-      <c r="L90" s="4" t="inlineStr"/>
-      <c r="M90" s="4" t="n"/>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L90" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M90" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N90" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4840,11 +6020,31 @@
       <c r="H91" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I91" s="4" t="n"/>
-      <c r="J91" s="4" t="n"/>
-      <c r="K91" s="4" t="n"/>
-      <c r="L91" s="4" t="inlineStr"/>
-      <c r="M91" s="4" t="n"/>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K91" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L91" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M91" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N91" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4882,11 +6082,31 @@
       <c r="H92" s="5" t="n">
         <v>-0.3321033210332103</v>
       </c>
-      <c r="I92" s="4" t="n"/>
-      <c r="J92" s="4" t="n"/>
-      <c r="K92" s="4" t="n"/>
-      <c r="L92" s="4" t="inlineStr"/>
-      <c r="M92" s="4" t="n"/>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L92" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M92" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N92" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4924,11 +6144,31 @@
       <c r="H93" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I93" s="4" t="n"/>
-      <c r="J93" s="4" t="n"/>
-      <c r="K93" s="4" t="n"/>
-      <c r="L93" s="4" t="inlineStr"/>
-      <c r="M93" s="4" t="n"/>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K93" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L93" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M93" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N93" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -4966,11 +6206,31 @@
       <c r="H94" s="5" t="n">
         <v>-0.3321033210332103</v>
       </c>
-      <c r="I94" s="4" t="n"/>
-      <c r="J94" s="4" t="n"/>
-      <c r="K94" s="4" t="n"/>
-      <c r="L94" s="4" t="inlineStr"/>
-      <c r="M94" s="4" t="n"/>
+      <c r="I94" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L94" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M94" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N94" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5008,11 +6268,31 @@
       <c r="H95" s="5" t="n">
         <v>-0.3321033210332103</v>
       </c>
-      <c r="I95" s="4" t="n"/>
-      <c r="J95" s="4" t="n"/>
-      <c r="K95" s="4" t="n"/>
-      <c r="L95" s="4" t="inlineStr"/>
-      <c r="M95" s="4" t="n"/>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L95" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M95" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N95" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5050,11 +6330,31 @@
       <c r="H96" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I96" s="4" t="n"/>
-      <c r="J96" s="4" t="n"/>
-      <c r="K96" s="4" t="n"/>
-      <c r="L96" s="4" t="inlineStr"/>
-      <c r="M96" s="4" t="n"/>
+      <c r="I96" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L96" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M96" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N96" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5092,11 +6392,31 @@
       <c r="H97" s="5" t="n">
         <v>-0.3321033210332103</v>
       </c>
-      <c r="I97" s="4" t="n"/>
-      <c r="J97" s="4" t="n"/>
-      <c r="K97" s="4" t="n"/>
-      <c r="L97" s="4" t="inlineStr"/>
-      <c r="M97" s="4" t="n"/>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L97" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M97" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N97" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5134,11 +6454,31 @@
       <c r="H98" s="5" t="n">
         <v>-0.3321033210332103</v>
       </c>
-      <c r="I98" s="4" t="n"/>
-      <c r="J98" s="4" t="n"/>
-      <c r="K98" s="4" t="n"/>
-      <c r="L98" s="4" t="inlineStr"/>
-      <c r="M98" s="4" t="n"/>
+      <c r="I98" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L98" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M98" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N98" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5176,11 +6516,31 @@
       <c r="H99" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I99" s="4" t="n"/>
-      <c r="J99" s="4" t="n"/>
-      <c r="K99" s="4" t="n"/>
-      <c r="L99" s="4" t="inlineStr"/>
-      <c r="M99" s="4" t="n"/>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L99" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M99" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N99" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5218,11 +6578,31 @@
       <c r="H100" s="5" t="n">
         <v>-0.4531722054380665</v>
       </c>
-      <c r="I100" s="4" t="n"/>
-      <c r="J100" s="4" t="n"/>
-      <c r="K100" s="4" t="n"/>
-      <c r="L100" s="4" t="inlineStr"/>
-      <c r="M100" s="4" t="n"/>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L100" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M100" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N100" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5260,11 +6640,31 @@
       <c r="H101" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I101" s="4" t="n"/>
-      <c r="J101" s="4" t="n"/>
-      <c r="K101" s="4" t="n"/>
-      <c r="L101" s="4" t="inlineStr"/>
-      <c r="M101" s="4" t="n"/>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L101" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M101" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N101" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5302,11 +6702,31 @@
       <c r="H102" s="5" t="n">
         <v>-0.1846846846846847</v>
       </c>
-      <c r="I102" s="4" t="n"/>
-      <c r="J102" s="4" t="n"/>
-      <c r="K102" s="4" t="n"/>
-      <c r="L102" s="4" t="inlineStr"/>
-      <c r="M102" s="4" t="n"/>
+      <c r="I102" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L102" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M102" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N102" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5348,11 +6768,31 @@
       <c r="H103" s="5" t="n">
         <v>-0.701010101010101</v>
       </c>
-      <c r="I103" s="4" t="n"/>
-      <c r="J103" s="4" t="n"/>
-      <c r="K103" s="4" t="n"/>
-      <c r="L103" s="4" t="inlineStr"/>
-      <c r="M103" s="4" t="n"/>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L103" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M103" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N103" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5390,11 +6830,31 @@
       <c r="H104" s="5" t="n">
         <v>-0.552870090634441</v>
       </c>
-      <c r="I104" s="4" t="n"/>
-      <c r="J104" s="4" t="n"/>
-      <c r="K104" s="4" t="n"/>
-      <c r="L104" s="4" t="inlineStr"/>
-      <c r="M104" s="4" t="n"/>
+      <c r="I104" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J104" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K104" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L104" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M104" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="N104" s="4" t="inlineStr">
         <is>
           <t>Hayır</t>
@@ -5404,7 +6864,7 @@
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>Not:</t>
+          <t>Kapsam:</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -5413,9 +6873,22 @@
         </is>
       </c>
     </row>
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>Google Trends:</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>Trends sütunları yalnızca sayfada listelenen 30 başlık için doldurulmuştur. Kalan 73 başlıkta "-" işareti, verinin bulunamadığını değil ölçümün yapılmadığını göstermektedir. Google Trends her başlık için ayrı sorgu gerektirdiğinden ölçüm kapsamı bilinçli olarak sınırlı tutulmuştur; talep halinde tüm başlıklara genişletilebilir.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B106:H106"/>
+  <mergeCells count="2">
+    <mergeCell ref="B107:I107"/>
+    <mergeCell ref="B106:I106"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12279,7 +13752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -12409,34 +13882,58 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Kat 1 / Kat 2 / Kat 3</t>
+          <t>Trends sütunlarında "-"</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Özdilekteyim kategori ağacının sırasıyla ana, alt ve detay seviyeleri.</t>
+          <t>İlgili başlık için Google Trends ölçümü yapılmadığını gösterir. Veri bulunamadığı anlamına gelmez. Trends her başlık için ayrı sorgu gerektirdiğinden ölçüm, sayfada listelenen başlıklarla sınırlı tutulmuştur.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Katalog Dışı Marka</t>
+          <t>Sayfada Listelendi</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Arama talebi bulunan ancak Özdilekteyim katalogunda yer almayan marka.</t>
+          <t>Başlığın rapor sayfasındaki tabloda gösterilip gösterilmediği. Google Trends ölçümü de bu başlıklar için yapılmıştır.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>Kat 1 / Kat 2 / Kat 3</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Özdilekteyim kategori ağacının sırasıyla ana, alt ve detay seviyeleri.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Katalog Dışı Marka</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Arama talebi bulunan ancak Özdilekteyim katalogunda yer almayan marka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Keskin Yükseliş</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Hacim sıralamasında geride kalan, ancak kendi yıl ortalamasına göre en belirgin ayrışan başlıklar. Zamanlama hassasiyeti yüksektir.</t>
         </is>

</xml_diff>

<commit_message>
Katalog dışı marka eşiği 15K'dan 5K'ya indi: 9 -> 12 marka
Katalog dışı 265 markanın 42'si büyüyor; 15K/ay hacim tabanı bunların
çoğunu büyümesi değil hacmi yüzünden eliyordu. Taban 5K'ya çekildi,
büyüme eşiği %20 olarak korundu. Listeye Altus (+%25), Intimissimi
(+%166) ve Selsil (+%71) girdi.

Yöntem satırı artık eşikleri sabit metin yerine LIMITS'ten okuyup açıkça
yazıyor; eşik değişince açıklama da değişiyor.

E-posta özeti hacme göre ilk 8'i gösterdiği için etkilenmedi. Excel'in
Katalog Dışı Markalar sayfası 12 satıra çıktı.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ozdilekteyim-eylul-2026-arama-talebi.xlsx
+++ b/ozdilekteyim-eylul-2026-arama-talebi.xlsx
@@ -7326,7 +7326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7501,13 +7501,61 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Altus</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>13671</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>0.2528639071330381</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Intimissimi</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>6066</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>1.659481183777859</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>1.13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Selsil</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>5569</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>0.7057172026544156</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Not:</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Özdilekteyim katalogunda yer almayan, son 12 ayda büyüyen markalardır.</t>
         </is>
@@ -7515,7 +7563,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>